<commit_message>
chore: update group schedule templates (matutino + vespertino)
</commit_message>
<xml_diff>
--- a/Template_Horarios_Grupos_Matutino.xlsx
+++ b/Template_Horarios_Grupos_Matutino.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\Customers\CBTis73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBAD704D-083D-4166-B089-081594DAC240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D55DB02B-3E64-4B82-A4D5-FE5E7AA548AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -511,13 +511,79 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="23" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="23" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="21" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -530,88 +596,22 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="21" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="23" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="23" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1416,12 +1416,12 @@
       <c r="A2" s="18"/>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
-      <c r="D2" s="68" t="s">
+      <c r="D2" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
       <c r="H2" s="1"/>
       <c r="I2" s="2"/>
     </row>
@@ -1429,12 +1429,12 @@
       <c r="A3" s="18"/>
       <c r="B3" s="20"/>
       <c r="C3" s="20"/>
-      <c r="D3" s="69" t="s">
+      <c r="D3" s="55" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
       <c r="H3" s="4"/>
       <c r="I3" s="5"/>
       <c r="J3">
@@ -1464,12 +1464,12 @@
       <c r="A5" s="18"/>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
-      <c r="D5" s="70"/>
-      <c r="E5" s="70"/>
-      <c r="F5" s="71" t="s">
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="71"/>
+      <c r="G5" s="57"/>
       <c r="H5" s="6"/>
       <c r="I5" s="5"/>
       <c r="J5">
@@ -1500,15 +1500,15 @@
       <c r="B7" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="72" t="s">
+      <c r="C7" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="73"/>
-      <c r="E7" s="74" t="s">
+      <c r="D7" s="59"/>
+      <c r="E7" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="74"/>
-      <c r="G7" s="74"/>
+      <c r="F7" s="60"/>
+      <c r="G7" s="60"/>
       <c r="H7" s="7"/>
       <c r="I7" s="5"/>
       <c r="J7">
@@ -1568,14 +1568,14 @@
     </row>
     <row r="10" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="19"/>
-      <c r="B10" s="78" t="s">
+      <c r="B10" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="56"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
       <c r="H10" s="9"/>
       <c r="I10" s="5"/>
       <c r="J10">
@@ -1591,12 +1591,12 @@
     </row>
     <row r="11" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="19"/>
-      <c r="B11" s="79"/>
-      <c r="C11" s="57"/>
-      <c r="D11" s="57"/>
-      <c r="E11" s="57"/>
-      <c r="F11" s="57"/>
-      <c r="G11" s="57"/>
+      <c r="B11" s="53"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
       <c r="H11" s="9"/>
       <c r="I11" s="5"/>
       <c r="J11">
@@ -1612,14 +1612,14 @@
     </row>
     <row r="12" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="19"/>
-      <c r="B12" s="75" t="s">
+      <c r="B12" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="56"/>
-      <c r="D12" s="56"/>
-      <c r="E12" s="56"/>
-      <c r="F12" s="56"/>
-      <c r="G12" s="56"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
       <c r="H12" s="9"/>
       <c r="I12" s="5"/>
       <c r="J12">
@@ -1635,12 +1635,12 @@
     </row>
     <row r="13" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="19"/>
-      <c r="B13" s="77"/>
-      <c r="C13" s="57"/>
-      <c r="D13" s="57"/>
-      <c r="E13" s="57"/>
-      <c r="F13" s="57"/>
-      <c r="G13" s="57"/>
+      <c r="B13" s="51"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
+      <c r="G13" s="49"/>
       <c r="H13" s="9"/>
       <c r="I13" s="5"/>
       <c r="J13">
@@ -1656,14 +1656,14 @@
     </row>
     <row r="14" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="19"/>
-      <c r="B14" s="78" t="s">
+      <c r="B14" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="63"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="64"/>
       <c r="H14" s="9"/>
       <c r="I14" s="5"/>
       <c r="J14">
@@ -1679,12 +1679,12 @@
     </row>
     <row r="15" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="19"/>
-      <c r="B15" s="79"/>
-      <c r="C15" s="57"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="57"/>
-      <c r="G15" s="64"/>
+      <c r="B15" s="53"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="49"/>
+      <c r="G15" s="65"/>
       <c r="H15" s="9"/>
       <c r="I15" s="5"/>
       <c r="J15">
@@ -1700,16 +1700,16 @@
     </row>
     <row r="16" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="19"/>
-      <c r="B16" s="76" t="s">
+      <c r="B16" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="65" t="s">
+      <c r="C16" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="66"/>
-      <c r="G16" s="67"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="67"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="68"/>
       <c r="H16" s="9"/>
       <c r="I16" s="5"/>
       <c r="J16">
@@ -1725,14 +1725,14 @@
     </row>
     <row r="17" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="19"/>
-      <c r="B17" s="75" t="s">
+      <c r="B17" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="61"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
+      <c r="C17" s="62"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="64"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="48"/>
       <c r="H17" s="9"/>
       <c r="I17" s="5"/>
       <c r="J17">
@@ -1748,12 +1748,12 @@
     </row>
     <row r="18" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="19"/>
-      <c r="B18" s="77"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="57"/>
-      <c r="E18" s="64"/>
-      <c r="F18" s="57"/>
-      <c r="G18" s="57"/>
+      <c r="B18" s="51"/>
+      <c r="C18" s="63"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="65"/>
+      <c r="F18" s="49"/>
+      <c r="G18" s="49"/>
       <c r="H18" s="9"/>
       <c r="I18" s="5"/>
       <c r="J18">
@@ -1769,14 +1769,14 @@
     </row>
     <row r="19" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="19"/>
-      <c r="B19" s="75" t="s">
+      <c r="B19" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="61"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
+      <c r="C19" s="62"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="48"/>
       <c r="H19" s="9"/>
       <c r="I19" s="5"/>
       <c r="J19">
@@ -1792,12 +1792,12 @@
     </row>
     <row r="20" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="19"/>
-      <c r="B20" s="77"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
+      <c r="B20" s="51"/>
+      <c r="C20" s="63"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
+      <c r="G20" s="49"/>
       <c r="H20" s="9"/>
       <c r="I20" s="5"/>
       <c r="J20">
@@ -1813,14 +1813,14 @@
     </row>
     <row r="21" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="19"/>
-      <c r="B21" s="75" t="s">
+      <c r="B21" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="56"/>
-      <c r="D21" s="56"/>
-      <c r="E21" s="56"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="56"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="48"/>
       <c r="H21" s="9"/>
       <c r="I21" s="5"/>
       <c r="J21">
@@ -1836,12 +1836,12 @@
     </row>
     <row r="22" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="19"/>
-      <c r="B22" s="77"/>
-      <c r="C22" s="57"/>
-      <c r="D22" s="57"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
       <c r="H22" s="9"/>
       <c r="I22" s="5"/>
       <c r="J22">
@@ -1857,14 +1857,14 @@
     </row>
     <row r="23" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="19"/>
-      <c r="B23" s="75" t="s">
+      <c r="B23" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="C23" s="56"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="56"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
+      <c r="C23" s="48"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
       <c r="H23" s="9"/>
       <c r="I23" s="5"/>
       <c r="J23">
@@ -1880,12 +1880,12 @@
     </row>
     <row r="24" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="19"/>
-      <c r="B24" s="77"/>
-      <c r="C24" s="57"/>
-      <c r="D24" s="57"/>
-      <c r="E24" s="57"/>
-      <c r="F24" s="57"/>
-      <c r="G24" s="57"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
       <c r="H24" s="9"/>
       <c r="I24" s="5"/>
       <c r="J24">
@@ -1901,14 +1901,14 @@
     </row>
     <row r="25" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="19"/>
-      <c r="B25" s="80" t="s">
+      <c r="B25" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="C25" s="56"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="56"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
       <c r="H25" s="9"/>
       <c r="I25" s="5"/>
       <c r="J25">
@@ -1924,12 +1924,12 @@
     </row>
     <row r="26" spans="1:15" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="19"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
+      <c r="B26" s="61"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
       <c r="H26" s="9"/>
       <c r="I26" s="5"/>
       <c r="J26">
@@ -2184,13 +2184,13 @@
       <c r="B39" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C39" s="58" t="s">
+      <c r="C39" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="59"/>
-      <c r="E39" s="59"/>
-      <c r="F39" s="59"/>
-      <c r="G39" s="60"/>
+      <c r="D39" s="70"/>
+      <c r="E39" s="70"/>
+      <c r="F39" s="70"/>
+      <c r="G39" s="71"/>
       <c r="H39" s="9"/>
       <c r="I39" s="5"/>
       <c r="J39">
@@ -2203,11 +2203,11 @@
     <row r="40" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="18"/>
       <c r="B40" s="27"/>
-      <c r="C40" s="53"/>
-      <c r="D40" s="54"/>
-      <c r="E40" s="54"/>
-      <c r="F40" s="54"/>
-      <c r="G40" s="55"/>
+      <c r="C40" s="75"/>
+      <c r="D40" s="76"/>
+      <c r="E40" s="76"/>
+      <c r="F40" s="76"/>
+      <c r="G40" s="77"/>
       <c r="H40" s="9"/>
       <c r="I40" s="5"/>
       <c r="J40">
@@ -2220,55 +2220,55 @@
     <row r="41" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="18"/>
       <c r="B41" s="27"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="48"/>
-      <c r="F41" s="48"/>
-      <c r="G41" s="49"/>
+      <c r="C41" s="78"/>
+      <c r="D41" s="79"/>
+      <c r="E41" s="79"/>
+      <c r="F41" s="79"/>
+      <c r="G41" s="80"/>
       <c r="H41" s="9"/>
       <c r="I41" s="5"/>
     </row>
     <row r="42" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="18"/>
       <c r="B42" s="27"/>
-      <c r="C42" s="47"/>
-      <c r="D42" s="48"/>
-      <c r="E42" s="48"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="49"/>
+      <c r="C42" s="78"/>
+      <c r="D42" s="79"/>
+      <c r="E42" s="79"/>
+      <c r="F42" s="79"/>
+      <c r="G42" s="80"/>
       <c r="H42" s="9"/>
       <c r="I42" s="5"/>
     </row>
     <row r="43" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="18"/>
       <c r="B43" s="27"/>
-      <c r="C43" s="47"/>
-      <c r="D43" s="48"/>
-      <c r="E43" s="48"/>
-      <c r="F43" s="48"/>
-      <c r="G43" s="49"/>
+      <c r="C43" s="78"/>
+      <c r="D43" s="79"/>
+      <c r="E43" s="79"/>
+      <c r="F43" s="79"/>
+      <c r="G43" s="80"/>
       <c r="H43" s="9"/>
       <c r="I43" s="5"/>
     </row>
     <row r="44" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="18"/>
       <c r="B44" s="27"/>
-      <c r="C44" s="47"/>
-      <c r="D44" s="48"/>
-      <c r="E44" s="48"/>
-      <c r="F44" s="48"/>
-      <c r="G44" s="49"/>
+      <c r="C44" s="78"/>
+      <c r="D44" s="79"/>
+      <c r="E44" s="79"/>
+      <c r="F44" s="79"/>
+      <c r="G44" s="80"/>
       <c r="H44" s="9"/>
       <c r="I44" s="5"/>
     </row>
     <row r="45" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="18"/>
       <c r="B45" s="27"/>
-      <c r="C45" s="47"/>
-      <c r="D45" s="48"/>
-      <c r="E45" s="48"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="49"/>
+      <c r="C45" s="78"/>
+      <c r="D45" s="79"/>
+      <c r="E45" s="79"/>
+      <c r="F45" s="79"/>
+      <c r="G45" s="80"/>
       <c r="I45" s="5"/>
       <c r="J45">
         <v>39</v>
@@ -2280,31 +2280,31 @@
     <row r="46" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="18"/>
       <c r="B46" s="27"/>
-      <c r="C46" s="47"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="48"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="49"/>
+      <c r="C46" s="78"/>
+      <c r="D46" s="79"/>
+      <c r="E46" s="79"/>
+      <c r="F46" s="79"/>
+      <c r="G46" s="80"/>
       <c r="I46" s="5"/>
     </row>
     <row r="47" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="18"/>
       <c r="B47" s="27"/>
-      <c r="C47" s="47"/>
-      <c r="D47" s="48"/>
-      <c r="E47" s="48"/>
-      <c r="F47" s="48"/>
-      <c r="G47" s="49"/>
+      <c r="C47" s="78"/>
+      <c r="D47" s="79"/>
+      <c r="E47" s="79"/>
+      <c r="F47" s="79"/>
+      <c r="G47" s="80"/>
       <c r="I47" s="5"/>
     </row>
     <row r="48" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="18"/>
       <c r="B48" s="27"/>
-      <c r="C48" s="47"/>
-      <c r="D48" s="48"/>
-      <c r="E48" s="48"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="49"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="79"/>
+      <c r="E48" s="79"/>
+      <c r="F48" s="79"/>
+      <c r="G48" s="80"/>
       <c r="I48" s="5"/>
       <c r="J48">
         <v>39</v>
@@ -2331,16 +2331,16 @@
     </row>
     <row r="50" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="18"/>
-      <c r="B50" s="50" t="s">
+      <c r="B50" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="C50" s="50"/>
-      <c r="D50" s="50"/>
-      <c r="E50" s="50" t="s">
+      <c r="C50" s="72"/>
+      <c r="D50" s="72"/>
+      <c r="E50" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="F50" s="50"/>
-      <c r="G50" s="50"/>
+      <c r="F50" s="72"/>
+      <c r="G50" s="72"/>
       <c r="I50" s="5"/>
       <c r="J50">
         <v>41</v>
@@ -2351,16 +2351,16 @@
     </row>
     <row r="51" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="18"/>
-      <c r="B51" s="51" t="s">
+      <c r="B51" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="C51" s="51"/>
-      <c r="D51" s="51"/>
-      <c r="E51" s="51" t="s">
+      <c r="C51" s="73"/>
+      <c r="D51" s="73"/>
+      <c r="E51" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="F51" s="51"/>
-      <c r="G51" s="51"/>
+      <c r="F51" s="73"/>
+      <c r="G51" s="73"/>
       <c r="I51" s="5"/>
       <c r="J51">
         <v>42</v>
@@ -2403,16 +2403,16 @@
     </row>
     <row r="54" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="18"/>
-      <c r="B54" s="50" t="s">
+      <c r="B54" s="72" t="s">
         <v>20</v>
       </c>
-      <c r="C54" s="50"/>
-      <c r="D54" s="50"/>
-      <c r="E54" s="50" t="s">
+      <c r="C54" s="72"/>
+      <c r="D54" s="72"/>
+      <c r="E54" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="F54" s="50"/>
-      <c r="G54" s="50"/>
+      <c r="F54" s="72"/>
+      <c r="G54" s="72"/>
       <c r="H54" s="8"/>
       <c r="I54" s="5"/>
       <c r="J54">
@@ -2424,16 +2424,16 @@
     </row>
     <row r="55" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="18"/>
-      <c r="B55" s="51" t="s">
+      <c r="B55" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="C55" s="51"/>
-      <c r="D55" s="51"/>
-      <c r="E55" s="51" t="s">
+      <c r="C55" s="73"/>
+      <c r="D55" s="73"/>
+      <c r="E55" s="73" t="s">
         <v>22</v>
       </c>
-      <c r="F55" s="51"/>
-      <c r="G55" s="51"/>
+      <c r="F55" s="73"/>
+      <c r="G55" s="73"/>
       <c r="H55" s="8"/>
       <c r="I55" s="5"/>
       <c r="J55">
@@ -2447,12 +2447,12 @@
       <c r="A56" s="18"/>
       <c r="B56" s="29"/>
       <c r="C56" s="29"/>
-      <c r="D56" s="52" t="s">
+      <c r="D56" s="74" t="s">
         <v>26</v>
       </c>
-      <c r="E56" s="52"/>
-      <c r="F56" s="52"/>
-      <c r="G56" s="52"/>
+      <c r="E56" s="74"/>
+      <c r="F56" s="74"/>
+      <c r="G56" s="74"/>
       <c r="H56" s="8"/>
       <c r="I56" s="5"/>
       <c r="J56">
@@ -2523,34 +2523,28 @@
     </row>
   </sheetData>
   <mergeCells count="66">
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="D3:G3"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="E55:G55"/>
+    <mergeCell ref="D56:G56"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="E50:G50"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="E54:G54"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B19:B20"/>
     <mergeCell ref="F14:F15"/>
     <mergeCell ref="G23:G24"/>
     <mergeCell ref="G25:G26"/>
@@ -2567,28 +2561,34 @@
     <mergeCell ref="C14:C15"/>
     <mergeCell ref="D14:D15"/>
     <mergeCell ref="E14:E15"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="B51:D51"/>
-    <mergeCell ref="E51:G51"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="E54:G54"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="E55:G55"/>
-    <mergeCell ref="D56:G56"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="D3:G3"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="G12:G13"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup scale="92" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>